<commit_message>
feat: update booking templates with new versions
</commit_message>
<xml_diff>
--- a/client/public/booking-empty-upload-template.xlsx
+++ b/client/public/booking-empty-upload-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marinljoljic/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marinljoljic/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA25927B-B920-0C4B-BD85-21814DAC1DB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2569FF7-86E9-2342-A517-01A6B2A39BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="600" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,10 +40,10 @@
     <t>End Date</t>
   </si>
   <si>
-    <t>Frequency</t>
-  </si>
-  <si>
     <t>Modality</t>
+  </si>
+  <si>
+    <t>Rounds</t>
   </si>
 </sst>
 </file>
@@ -431,7 +431,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -446,7 +446,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>